<commit_message>
feat: add student and family account access
</commit_message>
<xml_diff>
--- a/uploads/学生导入模板.xlsx
+++ b/uploads/学生导入模板.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,6 +487,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>职责</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>手机号</t>
         </is>
       </c>
     </row>

</xml_diff>